<commit_message>
fix: crypto dedup key → date-only, 1 row per day
</commit_message>
<xml_diff>
--- a/data/formulasi_pakan_ternak.xlsx
+++ b/data/formulasi_pakan_ternak.xlsx
@@ -2542,7 +2542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3107,37 +3107,6 @@
       <c r="A21" t="n">
         <v>1</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Jagung Pipilan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>35%</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>4896</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1714</v>
-      </c>
-      <c r="F21" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1.173</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.77</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3702,37 +3671,6 @@
       <c r="A39" t="n">
         <v>8</v>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Tepung Ikan</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>8023</v>
-      </c>
-      <c r="E39" t="n">
-        <v>321</v>
-      </c>
-      <c r="F39" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0.03</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4220,37 +4158,6 @@
       <c r="A57" t="n">
         <v>2</v>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Bungkil Kedelai</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>18%</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>7984</v>
-      </c>
-      <c r="E57" t="n">
-        <v>1437</v>
-      </c>
-      <c r="F57" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="G57" t="n">
-        <v>0.439</v>
-      </c>
-      <c r="H57" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="I57" t="n">
-        <v>0.117</v>
-      </c>
-      <c r="J57" t="n">
-        <v>1.08</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4782,175 +4689,181 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Catatan:</t>
+        </is>
+      </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>5032</v>
-      </c>
-      <c r="F75" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="G75" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="I75" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J75" t="n">
-        <v>7.6</v>
+          <t>Trimester akhir. Ca &amp; P tinggi untuk perkembangan janin.</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Catatan:</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Trimester akhir. Ca &amp; P tinggi untuk perkembangan janin.</t>
+          <t>📋 Sapi Laktasi Ringan</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>📋 Sapi Laktasi Ringan</t>
+          <t>Kebutuhan NRC:</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>PK min 14%</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>PK max 16%</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TDN 65%</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ME ≥ 2.6 Mcal/kg</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Ca ≥ 0.6%</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>P ≥ 0.4%</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>SK ≤ 22%</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Kebutuhan NRC:</t>
-        </is>
+      <c r="A78" t="n">
+        <v>1</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PK min 14%</t>
+          <t>Jagung Pipilan</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PK max 16%</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>TDN 65%</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>ME ≥ 2.6 Mcal/kg</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Ca ≥ 0.6%</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>P ≥ 0.4%</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>SK ≤ 22%</t>
-        </is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>4896</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1567</v>
+      </c>
+      <c r="F78" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1.072</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Jagung Pipilan</t>
+          <t>Bungkil Kedelai</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>4896</v>
+        <v>7984</v>
       </c>
       <c r="E79" t="n">
-        <v>1567</v>
+        <v>1118</v>
       </c>
       <c r="F79" t="n">
-        <v>26.88</v>
+        <v>4.9</v>
       </c>
       <c r="G79" t="n">
-        <v>1.072</v>
+        <v>0.342</v>
       </c>
       <c r="H79" t="n">
-        <v>0.006</v>
+        <v>0.048</v>
       </c>
       <c r="I79" t="n">
-        <v>0.09</v>
+        <v>0.091</v>
       </c>
       <c r="J79" t="n">
-        <v>0.7</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Bungkil Kedelai</t>
+          <t>Pollard</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>7984</v>
+        <v>4764</v>
       </c>
       <c r="E80" t="n">
-        <v>1118</v>
+        <v>381</v>
       </c>
       <c r="F80" t="n">
-        <v>4.9</v>
+        <v>1.2</v>
       </c>
       <c r="G80" t="n">
-        <v>0.342</v>
+        <v>0.164</v>
       </c>
       <c r="H80" t="n">
-        <v>0.048</v>
+        <v>0.01</v>
       </c>
       <c r="I80" t="n">
-        <v>0.091</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="J80" t="n">
-        <v>0.84</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Pollard</t>
+          <t>Bungkil Kacang Tanah</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4959,34 +4872,34 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>4764</v>
+        <v>8059</v>
       </c>
       <c r="E81" t="n">
-        <v>381</v>
+        <v>645</v>
       </c>
       <c r="F81" t="n">
-        <v>1.2</v>
+        <v>3.04</v>
       </c>
       <c r="G81" t="n">
-        <v>0.164</v>
+        <v>0.228</v>
       </c>
       <c r="H81" t="n">
-        <v>0.01</v>
+        <v>0.016</v>
       </c>
       <c r="I81" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.044</v>
       </c>
       <c r="J81" t="n">
-        <v>0.76</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Bungkil Kacang Tanah</t>
+          <t>Bungkil Kelapa</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4995,13 +4908,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>8059</v>
+        <v>8637</v>
       </c>
       <c r="E82" t="n">
-        <v>645</v>
+        <v>691</v>
       </c>
       <c r="F82" t="n">
-        <v>3.04</v>
+        <v>1.76</v>
       </c>
       <c r="G82" t="n">
         <v>0.228</v>
@@ -5010,7 +4923,7 @@
         <v>0.016</v>
       </c>
       <c r="I82" t="n">
-        <v>0.044</v>
+        <v>0.048</v>
       </c>
       <c r="J82" t="n">
         <v>0.96</v>
@@ -5018,113 +4931,77 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Bungkil Kelapa</t>
+          <t>Dedak Halus</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>8637</v>
+        <v>4006</v>
       </c>
       <c r="E83" t="n">
-        <v>691</v>
+        <v>140</v>
       </c>
       <c r="F83" t="n">
-        <v>1.76</v>
+        <v>0.46</v>
       </c>
       <c r="G83" t="n">
-        <v>0.228</v>
+        <v>0.063</v>
       </c>
       <c r="H83" t="n">
-        <v>0.016</v>
+        <v>0.003</v>
       </c>
       <c r="I83" t="n">
-        <v>0.048</v>
+        <v>0.047</v>
       </c>
       <c r="J83" t="n">
-        <v>0.96</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="n">
-        <v>9</v>
-      </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Dedak Halus</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>3.5%</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>4006</v>
+          <t>100.0%</t>
+        </is>
       </c>
       <c r="E84" t="n">
-        <v>140</v>
+        <v>5584</v>
       </c>
       <c r="F84" t="n">
-        <v>0.46</v>
+        <v>40.8</v>
       </c>
       <c r="G84" t="n">
-        <v>0.063</v>
+        <v>2.72</v>
       </c>
       <c r="H84" t="n">
-        <v>0.003</v>
+        <v>0.51</v>
       </c>
       <c r="I84" t="n">
-        <v>0.047</v>
+        <v>0.76</v>
       </c>
       <c r="J84" t="n">
-        <v>0.49</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Catatan:</t>
+        </is>
+      </c>
       <c r="B85" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="E85" t="n">
-        <v>5584</v>
-      </c>
-      <c r="F85" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="G85" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="H85" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="I85" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="J85" t="n">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Catatan:</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
         <is>
           <t>Laktasi 5-10L/hari. Protein &amp; Ca terjaga.</t>
         </is>
@@ -5754,37 +5631,6 @@
       <c r="A22" t="n">
         <v>1</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Jagung Pipilan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>4896</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1469</v>
-      </c>
-      <c r="F22" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="G22" t="n">
-        <v>1.005</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.66</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -6324,37 +6170,6 @@
     <row r="40">
       <c r="A40" t="n">
         <v>7</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Dedak Halus</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>6%</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>4006</v>
-      </c>
-      <c r="E40" t="n">
-        <v>240</v>
-      </c>
-      <c r="F40" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0.84</v>
       </c>
     </row>
     <row r="41">
@@ -7485,37 +7300,6 @@
       <c r="A23" t="n">
         <v>1</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Jagung Pipilan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>4896</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1860</v>
-      </c>
-      <c r="F23" t="n">
-        <v>31.92</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1.273</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.84</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -8112,11 +7896,6 @@
           <t>Status:</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>PK: ❌ | ME: ❌ | SK: ✅ | Ca: ❌ | P: ✅</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8633,37 +8412,6 @@
     <row r="60">
       <c r="A60" t="n">
         <v>8</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Ampas Tahu</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>3582</v>
-      </c>
-      <c r="E60" t="n">
-        <v>143</v>
-      </c>
-      <c r="F60" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="G60" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I60" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="J60" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="61">
@@ -9438,37 +9186,6 @@
       <c r="A23" t="n">
         <v>1</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Jagung Pipilan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>4896</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1860</v>
-      </c>
-      <c r="F23" t="n">
-        <v>31.92</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1.273</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.84</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10069,37 +9786,6 @@
       <c r="A42" t="n">
         <v>7</v>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Tepung Darah</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>8149</v>
-      </c>
-      <c r="E42" t="n">
-        <v>244</v>
-      </c>
-      <c r="F42" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="G42" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0.01</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -11290,37 +10976,6 @@
       <c r="A81" t="n">
         <v>9</v>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Ampas Tahu</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>3582</v>
-      </c>
-      <c r="E81" t="n">
-        <v>107</v>
-      </c>
-      <c r="F81" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="G81" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="H81" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="I81" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0.45</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11903,37 +11558,6 @@
     <row r="101">
       <c r="A101" t="n">
         <v>8</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Tepung Ikan</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="D101" t="n">
-        <v>8023</v>
-      </c>
-      <c r="E101" t="n">
-        <v>241</v>
-      </c>
-      <c r="F101" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="G101" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="H101" t="n">
-        <v>0.135</v>
-      </c>
-      <c r="I101" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="J101" t="n">
-        <v>0.02</v>
       </c>
     </row>
     <row r="102">
@@ -12541,36 +12165,6 @@
       <c r="A14" t="n">
         <v>8</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Ruminansia Kecil</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Kambing Konservasi</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>4324</v>
-      </c>
-      <c r="E14" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="F14" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>💲 Sedang</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -12758,36 +12352,6 @@
       <c r="A21" t="n">
         <v>14</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Non-Ruminansia (Babi)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Babi Grower (25-60kg)</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>5863</v>
-      </c>
-      <c r="E21" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="F21" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>💸 Mahal</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -12974,36 +12538,6 @@
     <row r="28">
       <c r="A28" t="n">
         <v>20</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Unggas</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broiler Finisher (25-35hr)</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>5903</v>
-      </c>
-      <c r="E28" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="F28" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>💸 Mahal</t>
-        </is>
       </c>
     </row>
     <row r="29">

</xml_diff>